<commit_message>
updated rosters and project teams
</commit_message>
<xml_diff>
--- a/teams-and-rosters/CS320-Sp24-102-roster.xlsx
+++ b/teams-and-rosters/CS320-Sp24-102-roster.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cygwin64\home\donha\cs320-spring2024\teams-and-rosters\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47290EBC-2AB4-423F-84E3-C4E5F52AE3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FB115C2-7185-46DC-8D70-3D9CA5160328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="667" windowWidth="26355" windowHeight="14858" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1103" yWindow="1073" windowWidth="23295" windowHeight="15127" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cs320-102-sp24-roster" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
   <si>
     <t>Major</t>
   </si>
@@ -58,12 +58,6 @@
     <t>Spencer</t>
   </si>
   <si>
-    <t>Loiseau</t>
-  </si>
-  <si>
-    <t>Andrew</t>
-  </si>
-  <si>
     <t>Mack</t>
   </si>
   <si>
@@ -74,12 +68,6 @@
   </si>
   <si>
     <t>Gabriel</t>
-  </si>
-  <si>
-    <t>Nelson</t>
-  </si>
-  <si>
-    <t>Alyssa</t>
   </si>
   <si>
     <t>Nielsen</t>
@@ -865,9 +853,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -905,7 +893,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1011,7 +999,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1153,7 +1141,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1161,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16.265625" customWidth="1"/>
@@ -1172,7 +1160,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="17" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B1" s="17"/>
       <c r="C1" s="17"/>
@@ -1180,10 +1168,10 @@
     </row>
     <row r="2" spans="1:4" s="2" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="13" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C2" s="13" t="s">
         <v>0</v>
@@ -1200,7 +1188,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>4</v>
@@ -1214,7 +1202,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>7</v>
@@ -1228,7 +1216,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>7</v>
@@ -1242,7 +1230,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>7</v>
@@ -1256,10 +1244,10 @@
         <v>13</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
@@ -1270,10 +1258,10 @@
         <v>15</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
@@ -1284,10 +1272,10 @@
         <v>17</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
@@ -1298,57 +1286,29 @@
         <v>19</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>4</v>
+      <c r="C11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A12" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A13" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
-    <row r="21" spans="4:4" x14ac:dyDescent="0.45">
-      <c r="D21" s="3"/>
+    <row r="12" spans="1:4" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
+    <row r="19" spans="4:4" x14ac:dyDescent="0.45">
+      <c r="D19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>